<commit_message>
Added readme to hour log
</commit_message>
<xml_diff>
--- a/DTT-Assessment-Hour-Log Kevin Bunk.xlsx
+++ b/DTT-Assessment-Hour-Log Kevin Bunk.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\DTT Assessment - Unity - 2023\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Desktop\Programming\Unity\DTT-Assessment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FF0247-01ED-4450-B425-281D29A3B926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92C836EC-BD9E-4C2A-B7E3-A9895311D394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="3525" windowWidth="21840" windowHeight="13740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="67">
   <si>
     <t>Subject</t>
   </si>
@@ -246,6 +246,15 @@
   <si>
     <t>Created a basic user manual with gifs for users who want to use it to generate their own mazes</t>
   </si>
+  <si>
+    <t>Created README</t>
+  </si>
+  <si>
+    <t>28/12/2025</t>
+  </si>
+  <si>
+    <t>Created a readme to the GitHub to help with the setup of the project</t>
+  </si>
 </sst>
 </file>
 
@@ -254,7 +263,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color indexed="8"/>
@@ -337,6 +346,12 @@
       <sz val="12"/>
       <color theme="10"/>
       <name val="Verdana"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Open Sans"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -556,7 +571,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -618,6 +633,15 @@
     </xf>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1877,7 +1901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultColWidth="6.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.69921875" style="1" customWidth="1"/>
@@ -2385,30 +2409,39 @@
       </c>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" spans="1:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="11"/>
-      <c r="B31" s="21"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="4"/>
+    <row r="31" spans="1:6" s="5" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="32">
+        <v>0.5</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B32" s="22">
-        <f>SUMIF(E4:E30,"&lt;&gt;x",B4:B30)</f>
-        <v>14.25</v>
-      </c>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
+      <c r="A32" s="11"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
       <c r="E32" s="3"/>
       <c r="F32" s="4"/>
     </row>
-    <row r="33" spans="1:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="6"/>
-      <c r="B33" s="23"/>
+    <row r="33" spans="1:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="22">
+        <f>SUMIF(E4:E31,"&lt;&gt;x",B4:B31)</f>
+        <v>14.25</v>
+      </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
@@ -2423,12 +2456,20 @@
       <c r="F34" s="4"/>
     </row>
     <row r="35" spans="1:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="24"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="9"/>
+      <c r="A35" s="6"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="4"/>
+    </row>
+    <row r="36" spans="1:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="7"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>